<commit_message>
docs: session close — backlog items 62-67, reference files w workflow
</commit_message>
<xml_diff>
--- a/solutions/bi/TraNag/TraNag_plan.xlsx
+++ b/solutions/bi/TraNag/TraNag_plan.xlsx
@@ -134,8 +134,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Dane_1" displayName="T_Dane_1" ref="A1:I209" headerRowCount="1">
-  <autoFilter ref="A1:I209"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Dane_1" displayName="T_Dane_1" ref="A1:I210" headerRowCount="1">
+  <autoFilter ref="A1:I210"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Kolejnosc"/>
     <tableColumn id="2" name="CDN_Pole"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I209"/>
+  <dimension ref="A1:I210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>CASE WHEN TrN_GIDTyp IN (2041,2045,1529) AND EXISTS(SELECT 1 FROM CDN.TraNag s2 WHERE s2.TrN_GIDNumer=TrN_SpiNumer AND s2.TrN_SpiTyp&lt;&gt;0) THEN '(Z)' WHEN TrN_Stan &amp; 2 = 2 AND TrN_GIDTyp IN (2041,2045,1529) THEN '(Z)' WHEN TrN_GenDokMag=-1 AND TrN_GIDTyp IN (1521,1529,1489) THEN '(A)' WHEN TrN_GenDokMag=-1 THEN '(s)' ELSE '' END + SKROT + '-' + CAST(TrN_TrNNumer AS VARCHAR) + '/' + RIGHT('0'+CAST(TrN_TrNMiesiac AS VARCHAR(2)),2) + '/' + RIGHT(CAST(TrN_TrNRok AS VARCHAR(4)),2) + CASE WHEN RTRIM(TrN_TrNSeria)='' THEN '' ELSE '/' + RTRIM(TrN_TrNSeria) END</t>
+          <t>CASE WHEN TrN_GIDTyp IN (2041,2045,1529) AND EXISTS(SELECT 1 FROM CDN.TraNag s WHERE s.TrN_SpiTyp=n.TrN_GIDTyp AND s.TrN_SpiNumer=n.TrN_GIDNumer AND ((n.TrN_GIDTyp=2041 AND s.TrN_GIDTyp=2009) OR (n.TrN_GIDTyp=2045 AND s.TrN_GIDTyp=2013) OR (n.TrN_GIDTyp=1529 AND s.TrN_GIDTyp=1497))) THEN '(Z)' WHEN TrN_Stan &amp; 2 = 2 AND TrN_GIDTyp IN (2041,2045,1529) THEN '(Z)' WHEN TrN_GenDokMag=-1 AND TrN_GIDTyp IN (1521,1529,1489) THEN '(A)' WHEN TrN_GenDokMag=-1 THEN '(s)' ELSE '' END + SKROT + '-' + CAST(TrN_TrNNumer AS VARCHAR) + '/' + RIGHT('0'+CAST(TrN_TrNMiesiac AS VARCHAR(2)),2) + '/' + RIGHT(CAST(TrN_TrNRok AS VARCHAR(4)),2) + CASE WHEN RTRIM(TrN_TrNSeria)='' THEN '' ELSE '/' + RTRIM(TrN_TrNSeria) END</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -5312,37 +5312,37 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>TrN_OpiLp</t>
+          <t>TrN_OpiNumer</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Lp opiekuna (stała)</t>
+          <t>Akronim opiekuna</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>RKUBOWSKI</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>POMIŃ</t>
+          <t>Opiekun_Akronim</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>CDN.PrcKarty Prc_Akronim (LEFT JOIN Prc_GIDNumer=TrN_OpiNumer, TrN_OpiTyp=944)</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Para lookup FK (pracownik/opiekun)</t>
         </is>
       </c>
     </row>
@@ -5352,12 +5352,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TrN_KarLp</t>
+          <t>TrN_OpiLp</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Lp karty (stała techniczna)</t>
+          <t>Lp opiekuna (stała)</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -5392,17 +5392,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>TrN_KnDTyp</t>
+          <t>TrN_KarLp</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Typ kontrahenta docelowego (32=Kontrahent)</t>
+          <t>Lp karty (stała techniczna)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>32, 0</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>N/D — redundantny przy KnDNumer</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Redundantny GIDTyp</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -5432,17 +5432,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>TrN_KnDFirma</t>
+          <t>TrN_KnDTyp</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ID firmy kontrahenta docelowego (stała)</t>
+          <t>Typ kontrahenta docelowego (32=Kontrahent)</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>32, 0</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>N/D — stały komponent GID</t>
+          <t>N/D — redundantny przy KnDNumer</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Stały komponent GID</t>
+          <t>Redundantny GIDTyp</t>
         </is>
       </c>
     </row>
@@ -5472,37 +5472,37 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>TrN_KnDNumer</t>
+          <t>TrN_KnDFirma</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>GID odbiorcy (kontrahenta docelowego)</t>
+          <t>ID firmy kontrahenta docelowego (stała)</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>0, 157, 277, ...</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>ID_Odbiorcy</t>
+          <t>POMIŃ</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>CASE WHEN TrN_KnDNumer=0 THEN NULL ELSE TrN_KnDNumer END</t>
+          <t>N/D — stały komponent GID</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Tak</t>
+          <t>Nie</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Kontrahent docelowy (odbiorca faktury gdy różny od płatnika) — JOIN do KntKarty</t>
+          <t>Stały komponent GID</t>
         </is>
       </c>
     </row>
@@ -5517,22 +5517,22 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Akronim odbiorcy</t>
+          <t>GID odbiorcy (kontrahenta docelowego)</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>ABCDE</t>
+          <t>0, 157, 277, ...</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Odbiorca_Akronim</t>
+          <t>ID_Odbiorcy</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>CDN.KntKarty Knt_Akronim (LEFT JOIN na TrN_KnDNumer, TrN_KnDTyp=32)</t>
+          <t>CASE WHEN TrN_KnDNumer=0 THEN NULL ELSE TrN_KnDNumer END</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Para lookup FK</t>
+          <t>Kontrahent docelowy (odbiorca faktury gdy różny od płatnika) — JOIN do KntKarty</t>
         </is>
       </c>
     </row>
@@ -5557,22 +5557,22 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Nazwa odbiorcy</t>
+          <t>Akronim odbiorcy</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Jan Kowalski</t>
+          <t>ABCDE</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Odbiorca_Nazwa</t>
+          <t>Odbiorca_Akronim</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>CDN.KntKarty Knt_Nazwa1</t>
+          <t>CDN.KntKarty Knt_Akronim (LEFT JOIN na TrN_KnDNumer, TrN_KnDTyp=32)</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -5592,37 +5592,37 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>TrN_KnDLp</t>
+          <t>TrN_KnDNumer</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Lp kontrahenta docelowego (stała)</t>
+          <t>Nazwa odbiorcy</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>Jan Kowalski</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>POMIŃ</t>
+          <t>Odbiorca_Nazwa</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>CDN.KntKarty Knt_Nazwa1</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Para lookup FK</t>
         </is>
       </c>
     </row>
@@ -5632,37 +5632,37 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>TrN_FormaNr</t>
+          <t>TrN_KnDLp</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Forma płatności</t>
+          <t>Lp kontrahenta docelowego (stała)</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>10=Gotówka, 20=Przelew, 30=Kredyt, 40=Czek, 50=Karta, 60=Inne</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Forma_Platnosci</t>
+          <t>POMIŃ</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>CASE WHEN TrN_FormaNr=10 THEN 'Gotówka' WHEN TrN_FormaNr=20 THEN 'Przelew' WHEN TrN_FormaNr=30 THEN 'Kredyt' WHEN TrN_FormaNr=40 THEN 'Czek' WHEN TrN_FormaNr=50 THEN 'Karta' WHEN TrN_FormaNr=60 THEN 'Inne' WHEN TrN_FormaNr=0 THEN NULL ELSE 'Użytkownika (' + CAST(TrN_FormaNr AS VARCHAR(5)) + ')' END</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Tak</t>
+          <t>Nie</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Forma płatności — analiza struktury płatności; gotówka vs przelew vs karta</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -5672,27 +5672,27 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>TrN_Rabat</t>
+          <t>TrN_FormaNr</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Rabat globalny dokumentu (%)</t>
+          <t>Forma płatności</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>0.00, 3.00, 10.00, 20.00</t>
+          <t>10=Gotówka, 20=Przelew, 30=Kredyt, 40=Czek, 50=Karta, 60=Inne</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Rabat_Proc</t>
+          <t>Forma_Platnosci</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>TrN_Rabat</t>
+          <t>CASE WHEN TrN_FormaNr=10 THEN 'Gotówka' WHEN TrN_FormaNr=20 THEN 'Przelew' WHEN TrN_FormaNr=30 THEN 'Kredyt' WHEN TrN_FormaNr=40 THEN 'Czek' WHEN TrN_FormaNr=50 THEN 'Karta' WHEN TrN_FormaNr=60 THEN 'Inne' WHEN TrN_FormaNr=0 THEN NULL ELSE 'Użytkownika (' + CAST(TrN_FormaNr AS VARCHAR(5)) + ')' END</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Procent rabatu — analiza polityki rabatowej per kontrahent/segment</t>
+          <t>Forma płatności — analiza struktury płatności; gotówka vs przelew vs karta</t>
         </is>
       </c>
     </row>
@@ -5712,37 +5712,37 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>TrN_RabatW</t>
+          <t>TrN_Rabat</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Rabat kwotowy (stała=0 lub distinct=1)</t>
+          <t>Rabat globalny dokumentu (%)</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.00, 3.00, 10.00, 20.00</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>POMIŃ</t>
+          <t>Rabat_Proc</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała wg listy stałych)</t>
+          <t>TrN_Rabat</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1; rabat kwotowy zawsze 0</t>
+          <t>Procent rabatu — analiza polityki rabatowej per kontrahent/segment</t>
         </is>
       </c>
     </row>
@@ -5752,37 +5752,37 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>TrN_CenaSpr</t>
+          <t>TrN_RabatW</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Numer ceny domyślnej dla transakcji</t>
+          <t>Rabat kwotowy (stała=0 lub distinct=1)</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>1, 2, 3, 4, 5, 6, ...</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Nr_Cennika</t>
+          <t>POMIŃ</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>TrN_CenaSpr</t>
+          <t>N/D — distinct=1 (stała wg listy stałych)</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Tak</t>
+          <t>Nie</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Poziom cennika zastosowany na dokumencie — analiza zastosowania cen</t>
+          <t>Stała techniczna — distinct=1; rabat kwotowy zawsze 0</t>
         </is>
       </c>
     </row>
@@ -5792,27 +5792,27 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>TrN_NettoP</t>
+          <t>TrN_CenaSpr</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Wartość netto (przychód / dotyczy też MM)</t>
+          <t>Numer ceny domyślnej dla transakcji</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>0.00, 6.48, 15.00, ...</t>
+          <t>1, 2, 3, 4, 5, 6, ...</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Wartosc_Netto_Przychod</t>
+          <t>Nr_Cennika</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>TrN_NettoP</t>
+          <t>TrN_CenaSpr</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Kwota netto przychodów — główna miara obrotowa dla PW/PZ/MMP</t>
+          <t>Poziom cennika zastosowany na dokumencie — analiza zastosowania cen</t>
         </is>
       </c>
     </row>
@@ -5832,27 +5832,27 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>TrN_NettoR</t>
+          <t>TrN_NettoP</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Wartość netto (rozchód / dotyczy też MM)</t>
+          <t>Wartość netto (przychód / dotyczy też MM)</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>0.00, 4.07, 8.94, ...</t>
+          <t>0.00, 6.48, 15.00, ...</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Wartosc_Netto_Rozchod</t>
+          <t>Wartosc_Netto_Przychod</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>TrN_NettoR</t>
+          <t>TrN_NettoP</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Kwota netto rozchodów — główna miara obrotowa dla WZ/RW/MMW/FS/FZ</t>
+          <t>Kwota netto przychodów — główna miara obrotowa dla PW/PZ/MMP</t>
         </is>
       </c>
     </row>
@@ -5872,27 +5872,27 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>TrN_WartoscWal</t>
+          <t>TrN_NettoR</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Wartość walutowa dokumentu (netto, dla eksportu)</t>
+          <t>Wartość netto (rozchód / dotyczy też MM)</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>0.00, 1007.72</t>
+          <t>0.00, 4.07, 8.94, ...</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Wartosc_Walutowa</t>
+          <t>Wartosc_Netto_Rozchod</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>TrN_WartoscWal</t>
+          <t>TrN_NettoR</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Wartość w walucie obcej — analiza eksportu i transakcji walutowych</t>
+          <t>Kwota netto rozchodów — główna miara obrotowa dla WZ/RW/MMW/FS/FZ</t>
         </is>
       </c>
     </row>
@@ -5912,27 +5912,27 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>TrN_WartoscDPPrzed</t>
+          <t>TrN_WartoscWal</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Wartość przed deprecjacją</t>
+          <t>Wartość walutowa dokumentu (netto, dla eksportu)</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.00, 1007.72</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Wartosc_Przed_Deprecjacja</t>
+          <t>Wartosc_Walutowa</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>TrN_WartoscDPPrzed</t>
+          <t>TrN_WartoscWal</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Deprecjacje — wartość przed; istotna dla 5 rekordów typu DP</t>
+          <t>Wartość w walucie obcej — analiza eksportu i transakcji walutowych</t>
         </is>
       </c>
     </row>
@@ -5952,27 +5952,27 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>TrN_WartoscDPPo</t>
+          <t>TrN_WartoscDPPrzed</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Wartość po deprecjacji</t>
+          <t>Wartość przed deprecjacją</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>nan/0.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Wartosc_Po_Deprecjacji</t>
+          <t>Wartosc_Przed_Deprecjacja</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>TrN_WartoscDPPo</t>
+          <t>TrN_WartoscDPPrzed</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Deprecjacje — wartość po; istotna dla 5 rekordów typu DP</t>
+          <t>Deprecjacje — wartość przed; istotna dla 5 rekordów typu DP</t>
         </is>
       </c>
     </row>
@@ -5992,27 +5992,27 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>TrN_Waluta</t>
+          <t>TrN_WartoscDPPo</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Symbol waluty</t>
+          <t>Wartość po deprecjacji</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>PLN, EUR, USD</t>
+          <t>nan/0.00</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Waluta</t>
+          <t>Wartosc_Po_Deprecjacji</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>TrN_Waluta</t>
+          <t>TrN_WartoscDPPo</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Waluta dokumentu — filtrowanie transakcji walutowych, analiza eksportu</t>
+          <t>Deprecjacje — wartość po; istotna dla 5 rekordów typu DP</t>
         </is>
       </c>
     </row>
@@ -6032,27 +6032,27 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>TrN_KursL</t>
+          <t>TrN_Waluta</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Licznik kursu walutowego</t>
+          <t>Symbol waluty</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>1.00, 402.04, 428.45, ...</t>
+          <t>PLN, EUR, USD</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Kurs_Walutowy</t>
+          <t>Waluta</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>CASE WHEN TrN_Waluta='PLN' THEN NULL ELSE CAST(TrN_KursL AS DECIMAL(10,4)) / CAST(NULLIF(TrN_KursM,0) AS DECIMAL(10,4)) END</t>
+          <t>TrN_Waluta</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Kurs wymiany (L/M) — analiza transakcji walutowych; PLN › NULL</t>
+          <t>Waluta dokumentu — filtrowanie transakcji walutowych, analiza eksportu</t>
         </is>
       </c>
     </row>
@@ -6072,37 +6072,37 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>TrN_KursM</t>
+          <t>TrN_KursL</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Mianownik kursu walutowego</t>
+          <t>Licznik kursu walutowego</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>1, 100</t>
+          <t>1.00, 402.04, 428.45, ...</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>POMIŃ</t>
+          <t>Kurs_Walutowy</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>N/D — wbudowany w kolumnę Kurs_Walutowy (L/M)</t>
+          <t>CASE WHEN TrN_Waluta='PLN' THEN NULL ELSE CAST(TrN_KursL AS DECIMAL(10,4)) / CAST(NULLIF(TrN_KursM,0) AS DECIMAL(10,4)) END</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Składnik kursu — zawarty w transformacji TrN_KursL; eksponowanie osobno zbędne</t>
+          <t>Kurs wymiany (L/M) — analiza transakcji walutowych; PLN › NULL</t>
         </is>
       </c>
     </row>
@@ -6112,17 +6112,17 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>TrN_KursLPierw</t>
+          <t>TrN_KursM</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Licznik kursu pierwotnego</t>
+          <t>Mianownik kursu walutowego</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>nan (brak danych)</t>
+          <t>1, 100</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>N/D — sample=nan; brak danych w bazie</t>
+          <t>N/D — wbudowany w kolumnę Kurs_Walutowy (L/M)</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>Brak danych w środowisku; brak wartości analitycznej</t>
+          <t>Składnik kursu — zawarty w transformacji TrN_KursL; eksponowanie osobno zbędne</t>
         </is>
       </c>
     </row>
@@ -6152,12 +6152,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>TrN_KursMPierw</t>
+          <t>TrN_KursLPierw</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Mianownik kursu pierwotnego</t>
+          <t>Licznik kursu pierwotnego</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -6192,37 +6192,37 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>TrN_VatTyp</t>
+          <t>TrN_KursMPierw</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Typ rejestru VAT</t>
+          <t>Mianownik kursu pierwotnego</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>0, 1=rejestr zakupu, 2=rejestr sprzedaży</t>
+          <t>nan (brak danych)</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Rejestr_VAT</t>
+          <t>POMIŃ</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>CASE TrN_VatTyp WHEN 1 THEN 'Zakup' WHEN 2 THEN 'Sprzedaż' WHEN 0 THEN NULL ELSE CAST(TrN_VatTyp AS VARCHAR(5)) END</t>
+          <t>N/D — sample=nan; brak danych w bazie</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Tak</t>
+          <t>Nie</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Rejestr VAT — kategoryzacja dokumentu dla analizy podatkowej</t>
+          <t>Brak danych w środowisku; brak wartości analitycznej</t>
         </is>
       </c>
     </row>
@@ -6232,27 +6232,27 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>TrN_FlagaNB</t>
+          <t>TrN_VatTyp</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Naliczanie VAT — netto (N) lub brutto (B)</t>
+          <t>Typ rejestru VAT</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>N, B</t>
+          <t>0, 1=rejestr zakupu, 2=rejestr sprzedaży</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>VAT_Od</t>
+          <t>Rejestr_VAT</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>CASE TrN_FlagaNB WHEN 'N' THEN 'Od netto' WHEN 'B' THEN 'Od brutto' ELSE TrN_FlagaNB END</t>
+          <t>CASE TrN_VatTyp WHEN 1 THEN 'Zakup' WHEN 2 THEN 'Sprzedaż' WHEN 0 THEN NULL ELSE CAST(TrN_VatTyp AS VARCHAR(5)) END</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>Metoda naliczania VAT — wpływa na kwoty; istotne przy analizie marży</t>
+          <t>Rejestr VAT — kategoryzacja dokumentu dla analizy podatkowej</t>
         </is>
       </c>
     </row>
@@ -6272,27 +6272,27 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>TrN_Platnosci</t>
+          <t>TrN_FlagaNB</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Czy dokument generuje płatności</t>
+          <t>Naliczanie VAT — netto (N) lub brutto (B)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>0=Nie, 1=Tak</t>
+          <t>N, B</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Jest_Platnosc</t>
+          <t>VAT_Od</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>CASE TrN_Platnosci WHEN 1 THEN 'Tak' WHEN 0 THEN 'Nie' ELSE CAST(TrN_Platnosci AS VARCHAR(3)) END</t>
+          <t>CASE TrN_FlagaNB WHEN 'N' THEN 'Od netto' WHEN 'B' THEN 'Od brutto' ELSE TrN_FlagaNB END</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Flaga płatności — segmentacja dokumentów z rozrachunkami</t>
+          <t>Metoda naliczania VAT — wpływa na kwoty; istotne przy analizie marży</t>
         </is>
       </c>
     </row>
@@ -6312,37 +6312,37 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>TrN_Wyslano</t>
+          <t>TrN_Platnosci</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Flaga wysłania (stała techniczna)</t>
+          <t>Czy dokument generuje płatności</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>0=Nie, 1=Tak</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>POMIŃ</t>
+          <t>Jest_Platnosc</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>CASE TrN_Platnosci WHEN 1 THEN 'Tak' WHEN 0 THEN 'Nie' ELSE CAST(TrN_Platnosci AS VARCHAR(3)) END</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Flaga płatności — segmentacja dokumentów z rozrachunkami</t>
         </is>
       </c>
     </row>
@@ -6352,37 +6352,37 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>TrN_DokumentObcy</t>
+          <t>TrN_Wyslano</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Numer dokumentu obcego (faktura dostawcy lub własny sformatowany)</t>
+          <t>Flaga wysłania (stała techniczna)</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>WZK-26/11/23/SPKRK, numer FZ ...</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Nr_Dokumentu_Obcego</t>
+          <t>POMIŃ</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>TrN_DokumentObcy</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Tak</t>
+          <t>Nie</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Numer nadany przez dostawcę (FZ/PZ) lub własny sformatowany — wyszukiwanie po numerze faktury dostawcy</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -6392,37 +6392,37 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>TrN_Intrastat</t>
+          <t>TrN_DokumentObcy</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Ująć w Intrastat (0=Nie, 1=Przywóz, 2=Wywóz)</t>
+          <t>Numer dokumentu obcego (faktura dostawcy lub własny sformatowany)</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>0, 1, 2</t>
+          <t>WZK-26/11/23/SPKRK, numer FZ ...</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>POMIŃ</t>
+          <t>Nr_Dokumentu_Obcego</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>N/D — is_useful=Nie</t>
+          <t>TrN_DokumentObcy</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Intrastat — is_useful=Nie; pole dla deklaracji statystycznych, nie dla analizy obrotu</t>
+          <t>Numer nadany przez dostawcę (FZ/PZ) lub własny sformatowany — wyszukiwanie po numerze faktury dostawcy</t>
         </is>
       </c>
     </row>
@@ -6432,37 +6432,37 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>TrN_IncotermsSymbol</t>
+          <t>TrN_Intrastat</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Warunki dostawy wg Incoterms</t>
+          <t>Ująć w Intrastat (0=Nie, 1=Przywóz, 2=Wywóz)</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>EXW, FOB, CIF, ...</t>
+          <t>0, 1, 2</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Incoterms</t>
+          <t>POMIŃ</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>NULLIF(RTRIM(TrN_IncotermsSymbol), '')</t>
+          <t>N/D — is_useful=Nie</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Tak</t>
+          <t>Nie</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>Incoterms — analiza warunków handlowych transakcji eksportowych</t>
+          <t>Intrastat — is_useful=Nie; pole dla deklaracji statystycznych, nie dla analizy obrotu</t>
         </is>
       </c>
     </row>
@@ -6472,37 +6472,37 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>TrN_IncotermsMiejsce</t>
+          <t>TrN_IncotermsSymbol</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Miejsce Incoterms (stała)</t>
+          <t>Warunki dostawy wg Incoterms</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>nan (brak danych)</t>
+          <t>EXW, FOB, CIF, ...</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>POMIŃ</t>
+          <t>Incoterms</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała w liście stałych)</t>
+          <t>NULLIF(RTRIM(TrN_IncotermsSymbol), '')</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Incoterms — analiza warunków handlowych transakcji eksportowych</t>
         </is>
       </c>
     </row>
@@ -6512,17 +6512,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>TrN_Waga</t>
+          <t>TrN_IncotermsMiejsce</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Waga netto (stała techniczna)</t>
+          <t>Miejsce Incoterms (stała)</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>nan (brak danych)</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>N/D — distinct=1 (stała w liście stałych)</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -6552,12 +6552,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>TrN_WagaBrutto</t>
+          <t>TrN_Waga</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Waga brutto (stała techniczna)</t>
+          <t>Waga netto (stała techniczna)</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -6592,12 +6592,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>TrN_NumerSAD</t>
+          <t>TrN_WagaBrutto</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Numer SAD (stała techniczna)</t>
+          <t>Waga brutto (stała techniczna)</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -6632,12 +6632,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>TrN_MiejsceZaladunku</t>
+          <t>TrN_NumerSAD</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Miejsce załadunku (stała techniczna)</t>
+          <t>Numer SAD (stała techniczna)</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -6672,12 +6672,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>TrN_MiejscePrzeznaczenia</t>
+          <t>TrN_MiejsceZaladunku</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Miejsce przeznaczenia (stała techniczna)</t>
+          <t>Miejsce załadunku (stała techniczna)</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -6712,12 +6712,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>TrN_RodzajTransportu</t>
+          <t>TrN_MiejscePrzeznaczenia</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Rodzaj transportu (stała techniczna)</t>
+          <t>Miejsce przeznaczenia (stała techniczna)</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -6752,12 +6752,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>TrN_InfoDlaUC</t>
+          <t>TrN_RodzajTransportu</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Info dla urzędu celnego (stała)</t>
+          <t>Rodzaj transportu (stała techniczna)</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -6792,17 +6792,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>TrN_KrajPrzezWys</t>
+          <t>TrN_InfoDlaUC</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Kraj przeznaczenia/wysyłki</t>
+          <t>Info dla urzędu celnego (stała)</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>IE, CN, PL, ...</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>N/D — is_useful=Nie</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>is_useful=Nie — kraj wysyłki; nie eksponujemy w widoku podstawowym</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -6832,17 +6832,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>TrN_Struktura</t>
+          <t>TrN_KrajPrzezWys</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Czy uwzględniać w strukturze sprzedaży</t>
+          <t>Kraj przeznaczenia/wysyłki</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>0, 1, 2</t>
+          <t>IE, CN, PL, ...</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>N/D — is_useful=? (niejasne); pole wewnętrzne struktury sprzedaży</t>
+          <t>N/D — is_useful=Nie</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Niejasne is_useful; pole nieanalityczne dla widoku obrotu; pomijamy</t>
+          <t>is_useful=Nie — kraj wysyłki; nie eksponujemy w widoku podstawowym</t>
         </is>
       </c>
     </row>
@@ -6872,17 +6872,17 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>TrN_Detal</t>
+          <t>TrN_Struktura</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Flaga sprzedaży detalicznej (stała)</t>
+          <t>Czy uwzględniać w strukturze sprzedaży</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>0, 1, 2</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -6892,7 +6892,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>N/D — is_useful=? (niejasne); pole wewnętrzne struktury sprzedaży</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Niejasne is_useful; pole nieanalityczne dla widoku obrotu; pomijamy</t>
         </is>
       </c>
     </row>
@@ -6912,37 +6912,37 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>TrN_DokTypJPK</t>
+          <t>TrN_Detal</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Kod grupy towaru JPK (GTU)</t>
+          <t>Flaga sprzedaży detalicznej (stała)</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>FP, RO, MK</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Kod_JPK</t>
+          <t>POMIŃ</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>NULLIF(RTRIM(TrN_DokTypJPK), '')</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Tak</t>
+          <t>Nie</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Kod JPK dokumentu (FP=faktura do paragonu, RO=raport, MK=metoda kasowa) — analiza typów dla JPK_V7</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -6952,37 +6952,37 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>TrN_KatDatyOP</t>
+          <t>TrN_DokTypJPK</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Kategoria daty obowiązku podatkowego</t>
+          <t>Kod grupy towaru JPK (GTU)</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>0, 1, 2, 3, 11, 12, 13</t>
+          <t>FP, RO, MK</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>POMIŃ</t>
+          <t>Kod_JPK</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>N/D — is_useful=Nie</t>
+          <t>NULLIF(RTRIM(TrN_DokTypJPK), '')</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Nie</t>
+          <t>Tak</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Kategoria techniczna VAT — is_useful=Nie; brak wartości analitycznej dla widoku obrotu</t>
+          <t>Kod JPK dokumentu (FP=faktura do paragonu, RO=raport, MK=metoda kasowa) — analiza typów dla JPK_V7</t>
         </is>
       </c>
     </row>
@@ -6992,17 +6992,17 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>TrN_OCR</t>
+          <t>TrN_KatDatyOP</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Zaczytany przez OCR (0/1/2)</t>
+          <t>Kategoria daty obowiązku podatkowego</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>0, 1, 2</t>
+          <t>0, 1, 2, 3, 11, 12, 13</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -7022,7 +7022,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Metoda wprowadzenia — is_useful=Nie; brak wartości analitycznej</t>
+          <t>Kategoria techniczna VAT — is_useful=Nie; brak wartości analitycznej dla widoku obrotu</t>
         </is>
       </c>
     </row>
@@ -7032,17 +7032,17 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>TrN_Promocje</t>
+          <t>TrN_OCR</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Flaga promocji (stała techniczna)</t>
+          <t>Zaczytany przez OCR (0/1/2)</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>0, 1, 2</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -7052,7 +7052,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>N/D — is_useful=Nie</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -7062,7 +7062,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Metoda wprowadzenia — is_useful=Nie; brak wartości analitycznej</t>
         </is>
       </c>
     </row>
@@ -7072,12 +7072,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>TrN_DataOdb</t>
+          <t>TrN_Promocje</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Data odbioru (stała techniczna)</t>
+          <t>Flaga promocji (stała techniczna)</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -7112,12 +7112,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>TrN_PotwierdzenieOdbioru</t>
+          <t>TrN_DataOdb</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Potwierdzenie odbioru (stała techniczna)</t>
+          <t>Data odbioru (stała techniczna)</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -7152,17 +7152,17 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>TrN_RabatPromocyjnyGlobalny</t>
+          <t>TrN_PotwierdzenieOdbioru</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Rabat promocyjny globalny (stała)</t>
+          <t>Potwierdzenie odbioru (stała techniczna)</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -7172,7 +7172,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała); brak danych</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -7192,17 +7192,17 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>TrN_ZwroconoCalaIlosc</t>
+          <t>TrN_RabatPromocyjnyGlobalny</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Zwrócono całą ilość (stała)</t>
+          <t>Rabat promocyjny globalny (stała)</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>N/D — distinct=1 (stała); brak danych</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -7232,12 +7232,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>TrN_TerminRozliczeniaKaucji</t>
+          <t>TrN_ZwroconoCalaIlosc</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Termin rozliczenia kaucji (stała)</t>
+          <t>Zwrócono całą ilość (stała)</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -7272,12 +7272,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>TrN_OddZakazPAFA</t>
+          <t>TrN_TerminRozliczeniaKaucji</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Oddział zakaz PAFA (stała)</t>
+          <t>Termin rozliczenia kaucji (stała)</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -7312,12 +7312,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>TrN_WsSCHNumer</t>
+          <t>TrN_OddZakazPAFA</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Numer schematu WS (stała)</t>
+          <t>Oddział zakaz PAFA (stała)</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -7352,12 +7352,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>TrN_WsStosujSchemat</t>
+          <t>TrN_WsSCHNumer</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Czy stosować schemat WS (stała)</t>
+          <t>Numer schematu WS (stała)</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -7392,12 +7392,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>TrN_WsDziennik</t>
+          <t>TrN_WsStosujSchemat</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Dziennik WS (stała)</t>
+          <t>Czy stosować schemat WS (stała)</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -7432,12 +7432,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>TrN_WsStosujDziennik</t>
+          <t>TrN_WsDziennik</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Czy stosować dziennik WS (stała)</t>
+          <t>Dziennik WS (stała)</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -7472,12 +7472,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>TrN_PrjId</t>
+          <t>TrN_WsStosujDziennik</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>ID projektu (stała techniczna)</t>
+          <t>Czy stosować dziennik WS (stała)</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -7512,17 +7512,17 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>TrN_KnSTypD / TrN_KnSFirmaD / TrN_KnSNumerD / TrN_KnSLpD</t>
+          <t>TrN_PrjId</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>GID osoby kontrahenta docelowego (is_useful=brak)</t>
+          <t>ID projektu (stała techniczna)</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>N/D — is_useful puste; brak danych</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Puste w bazie (nan); brak wartości analitycznej</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -7552,12 +7552,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>TrN_KnSTypP / TrN_KnSFirmaP / TrN_KnSNumerP / TrN_KnSLpP</t>
+          <t>TrN_KnSTypD / TrN_KnSFirmaD / TrN_KnSNumerD / TrN_KnSLpD</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>GID osoby płatnika (is_useful=brak)</t>
+          <t>GID osoby kontrahenta docelowego (is_useful=brak)</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -7592,17 +7592,17 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>TrN_FrmNumer</t>
+          <t>TrN_KnSTypP / TrN_KnSFirmaP / TrN_KnSNumerP / TrN_KnSLpP</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Pieczątka (ID)</t>
+          <t>GID osoby płatnika (is_useful=brak)</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>1 (stała)</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -7612,7 +7612,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>N/D — is_useful=Nie; distinct=1 (stała)</t>
+          <t>N/D — is_useful puste; brak danych</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Stała techniczna — is_useful=Nie; distinct=1</t>
+          <t>Puste w bazie (nan); brak wartości analitycznej</t>
         </is>
       </c>
     </row>
@@ -7632,17 +7632,17 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>TrN_PrzywracajRezerwacje</t>
+          <t>TrN_FrmNumer</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Przywracaj rezerwacje (stała)</t>
+          <t>Pieczątka (ID)</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>1 (stała)</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>N/D — is_useful=Nie; distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -7662,7 +7662,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Stała techniczna — is_useful=Nie; distinct=1</t>
         </is>
       </c>
     </row>
@@ -7672,12 +7672,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>TrN_FormatkaCyr</t>
+          <t>TrN_PrzywracajRezerwacje</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Formatka Cyr (stała)</t>
+          <t>Przywracaj rezerwacje (stała)</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -7712,17 +7712,17 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>TrN_WtrID</t>
+          <t>TrN_FormatkaCyr</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>ID promocji wartościowej (brak danych)</t>
+          <t>Formatka Cyr (stała)</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>N/D — is_useful puste; brak danych (nan)</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -7742,7 +7742,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Brak danych w bazie; brak wartości analitycznej</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -7752,17 +7752,17 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>TrN_WtrProgID</t>
+          <t>TrN_WtrID</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>ID programu WTR (stała)</t>
+          <t>ID promocji wartościowej (brak danych)</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>N/D — is_useful puste; brak danych (nan)</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Brak danych w bazie; brak wartości analitycznej</t>
         </is>
       </c>
     </row>
@@ -7792,12 +7792,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>TrN_RodzajKor</t>
+          <t>TrN_WtrProgID</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Rodzaj korekty (stała)</t>
+          <t>ID programu WTR (stała)</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -7832,12 +7832,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>TrN_VatZDPeDNumer</t>
+          <t>TrN_RodzajKor</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Numer ZDP-eD VAT (stała)</t>
+          <t>Rodzaj korekty (stała)</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -7872,12 +7872,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>TrN_VatZDPeDLp</t>
+          <t>TrN_VatZDPeDNumer</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Lp ZDP-eD VAT (stała)</t>
+          <t>Numer ZDP-eD VAT (stała)</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -7912,12 +7912,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>TrN_DataDostawy</t>
+          <t>TrN_VatZDPeDLp</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Data dostawy (stała techniczna)</t>
+          <t>Lp ZDP-eD VAT (stała)</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -7952,12 +7952,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>TrN_WMS</t>
+          <t>TrN_DataDostawy</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Flaga WMS (stała techniczna)</t>
+          <t>Data dostawy (stała techniczna)</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -7992,17 +7992,17 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>TrN_VATNalOd</t>
+          <t>TrN_WMS</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>VAT naliczony od (stała)</t>
+          <t>Flaga WMS (stała techniczna)</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -8012,7 +8012,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała); is_useful puste</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -8032,12 +8032,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>TrN_OpeTypZM / TrN_OpeNumerZM / TrN_TStampZM</t>
+          <t>TrN_VATNalOd</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Operator zatwierdzający merytorycznie (ZM)</t>
+          <t>VAT naliczony od (stała)</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -8052,7 +8052,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>N/D — is_useful puste; brak danych (nan)</t>
+          <t>N/D — distinct=1 (stała); is_useful puste</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -8062,7 +8062,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>Brak danych w bazie; pola zatwierdzeń merytorycznych nieużywane</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -8072,12 +8072,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>TrN_OpeTypZFR / TrN_OpeNumerZFR / TrN_TStampZFR</t>
+          <t>TrN_OpeTypZM / TrN_OpeNumerZM / TrN_TStampZM</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Operator zatwierdzający formalno-rachunkowo (ZFR)</t>
+          <t>Operator zatwierdzający merytorycznie (ZM)</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -8102,7 +8102,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>Brak danych w bazie; pola zatwierdzeń nieużywane</t>
+          <t>Brak danych w bazie; pola zatwierdzeń merytorycznych nieużywane</t>
         </is>
       </c>
     </row>
@@ -8112,17 +8112,17 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>TrN_ZatwMerytorycznie</t>
+          <t>TrN_OpeTypZFR / TrN_OpeNumerZFR / TrN_TStampZFR</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Zatwierdzone merytorycznie (stała)</t>
+          <t>Operator zatwierdzający formalno-rachunkowo (ZFR)</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>stała</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -8132,7 +8132,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała)</t>
+          <t>N/D — is_useful puste; brak danych (nan)</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -8142,7 +8142,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1</t>
+          <t>Brak danych w bazie; pola zatwierdzeń nieużywane</t>
         </is>
       </c>
     </row>
@@ -8152,12 +8152,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>TrN_ZatwFormalnoRach</t>
+          <t>TrN_ZatwMerytorycznie</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Zatwierdzone formalno-rachunkowo (stała)</t>
+          <t>Zatwierdzone merytorycznie (stała)</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -8192,12 +8192,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>TrN_DataWplywuFA</t>
+          <t>TrN_ZatwFormalnoRach</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Data wpływu FA (stała)</t>
+          <t>Zatwierdzone formalno-rachunkowo (stała)</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -8232,12 +8232,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>TrN_PodzialPlatNiePytaj</t>
+          <t>TrN_DataWplywuFA</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Podział płatności nie pytaj (stała)</t>
+          <t>Data wpływu FA (stała)</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -8272,12 +8272,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>TrN_ProceduraUproszcz</t>
+          <t>TrN_PodzialPlatNiePytaj</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Procedura uproszczona (stała)</t>
+          <t>Podział płatności nie pytaj (stała)</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -8312,12 +8312,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>TrN_MPP</t>
+          <t>TrN_ProceduraUproszcz</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Mechanizm podzielonej płatności (stała)</t>
+          <t>Procedura uproszczona (stała)</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -8352,12 +8352,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>TrN_JestLimitCelowy</t>
+          <t>TrN_MPP</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Jest limit celowy (stała)</t>
+          <t>Mechanizm podzielonej płatności (stała)</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -8392,12 +8392,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>TrN_OplataSpozFlaga</t>
+          <t>TrN_JestLimitCelowy</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Opłata spożywcza (stała)</t>
+          <t>Jest limit celowy (stała)</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -8432,12 +8432,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>TrN_UmNId</t>
+          <t>TrN_OplataSpozFlaga</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>ID umowy (stała)</t>
+          <t>Opłata spożywcza (stała)</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -8472,12 +8472,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>TrN_ProceduraOSS</t>
+          <t>TrN_UmNId</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Procedura OSS (stała)</t>
+          <t>ID umowy (stała)</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -8512,12 +8512,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>TrN_RozliczacVIU</t>
+          <t>TrN_ProceduraOSS</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Rozliczać VIU (stała)</t>
+          <t>Procedura OSS (stała)</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -8552,12 +8552,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>TrN_KorektaVIU</t>
+          <t>TrN_RozliczacVIU</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Korekta VIU (stała)</t>
+          <t>Rozliczać VIU (stała)</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -8592,17 +8592,17 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>TrN_KrajWydania</t>
+          <t>TrN_KorektaVIU</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Skrót kraju wydania (is_useful=Nie)</t>
+          <t>Korekta VIU (stała)</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>brak danych</t>
+          <t>stała</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>N/D — is_useful=Nie; distinct=1 (stała)</t>
+          <t>N/D — distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -8622,7 +8622,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>Stała techniczna — is_useful=Nie</t>
+          <t>Stała techniczna — distinct=1</t>
         </is>
       </c>
     </row>
@@ -8632,12 +8632,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>TrN_KrajWydIdentPod</t>
+          <t>TrN_KrajWydania</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Identyfikator podatkowy kraju wydania (is_useful=Nie)</t>
+          <t>Skrót kraju wydania (is_useful=Nie)</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -8672,17 +8672,17 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>TrN_KrajWydIdentPodVAT</t>
+          <t>TrN_KrajWydIdentPod</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Czy ma numer VAT kraju wydania (is_useful=Nie)</t>
+          <t>Identyfikator podatkowy kraju wydania (is_useful=Nie)</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>brak danych</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -8712,12 +8712,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>TrN_KSeFWyslij</t>
+          <t>TrN_KrajWydIdentPodVAT</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Status wysyłki do KSeF (stała=0)</t>
+          <t>Czy ma numer VAT kraju wydania (is_useful=Nie)</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała=0); KSeF jeszcze nieobowiązkowy</t>
+          <t>N/D — is_useful=Nie; distinct=1 (stała)</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -8742,7 +8742,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>Stała techniczna — wszyscy 0; KSeF nieaktywny w firmie</t>
+          <t>Stała techniczna — is_useful=Nie</t>
         </is>
       </c>
     </row>
@@ -8752,17 +8752,17 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>TrN_KSeFNumerOrg</t>
+          <t>TrN_KSeFWyslij</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Nr KSeF oryginału (stała)</t>
+          <t>Status wysyłki do KSeF (stała=0)</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>brak danych</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>N/D — distinct=1 (stała); KSeF nieaktywny</t>
+          <t>N/D — distinct=1 (stała=0); KSeF jeszcze nieobowiązkowy</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -8782,7 +8782,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>Stała techniczna — distinct=1; KSeF nieaktywny</t>
+          <t>Stała techniczna — wszyscy 0; KSeF nieaktywny w firmie</t>
         </is>
       </c>
     </row>
@@ -8792,35 +8792,75 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
+          <t>TrN_KSeFNumerOrg</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Nr KSeF oryginału (stała)</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>brak danych</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>POMIŃ</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>N/D — distinct=1 (stała); KSeF nieaktywny</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Stała techniczna — distinct=1; KSeF nieaktywny</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
           <t>TrN_GodzinaWystawienia</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr">
+      <c r="C210" t="inlineStr">
         <is>
           <t>Godzina wystawienia dokumentu (is_useful=Nie)</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr">
+      <c r="D210" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr">
-        <is>
-          <t>POMIŃ</t>
-        </is>
-      </c>
-      <c r="F209" t="inlineStr">
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>POMIŃ</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
         <is>
           <t>N/D — is_useful=Nie</t>
         </is>
       </c>
-      <c r="G209" t="inlineStr">
-        <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H209" t="inlineStr">
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
         <is>
           <t>is_useful=Nie — brak wartości analitycznej</t>
         </is>

</xml_diff>